<commit_message>
Add all possible max-3 bundle generator
Co-authored-by: bassemmamdouh-crypto <bassemmamdouh-crypto@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bundle_planning_template.xlsx
+++ b/bundle_planning_template.xlsx
@@ -10,11 +10,13 @@
     <sheet name="Input_Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Scoring_Model" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Bundle_Recommendations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Logic" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="All_Possible_Bundles" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Logic" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scoring_Model'!$A$1:$Y$300</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bundle_Recommendations'!$A$1:$K$300</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All_Possible_Bundles'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +36,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -65,13 +70,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L300"/>
+  <dimension ref="A1:L301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1648,6 +1659,7 @@
     <row r="300">
       <c r="I300" s="2" t="n"/>
     </row>
+    <row r="301"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1659,7 +1671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y300"/>
+  <dimension ref="A1:Y301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32314,6 +32326,7 @@
         <v/>
       </c>
     </row>
+    <row r="301"/>
   </sheetData>
   <autoFilter ref="A1:Y300"/>
   <conditionalFormatting sqref="T2:T300">
@@ -46181,14 +46194,409 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="56" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>bundle_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>bundle_size</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>anchor_product_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>anchor_product_name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>item_2_product_id</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>item_2_product_name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>item_3_product_id</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>item_3_product_name</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>category_mix</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>bundle_priority_score</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>suggested_discount_%</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>B-000001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>P-2002</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Sea Salt Crackers</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>P-3001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Aloe Vera Gel 250ml</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Cross Category</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0.8500000000000001</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Moves one slow mover using one customer-attracting anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B-000002</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P-2002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sea Salt Crackers</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>P-2001</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Dry Fruit Mix 200g</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Same Category</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0.7375</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>0.09000000000000001</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Moves one slow mover using one customer-attracting anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>B-000003</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P-1001</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sparkling Water 330ml</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>P-3001</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Aloe Vera Gel 250ml</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cross Category</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0.7875000000000001</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Moves one slow mover using one customer-attracting anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B-000004</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>P-1001</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Sparkling Water 330ml</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>P-2001</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Dry Fruit Mix 200g</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Cross Category</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0.675</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>0.09000000000000001</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Moves one slow mover using one customer-attracting anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B-000005</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>P-2002</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sea Salt Crackers</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>P-3001</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Aloe Vera Gel 250ml</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P-2001</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Dry Fruit Mix 200g</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Mixed Category</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0.7875000000000001</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>0.09000000000000001</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Moves two slow movers with one anchor while keeping discount controlled</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B-000006</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>P-1001</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Sparkling Water 330ml</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>P-3001</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Aloe Vera Gel 250ml</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P-2001</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Dry Fruit Mix 200g</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Mixed Category</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0.7375</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0.09000000000000001</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Moves two slow movers with one anchor while keeping discount controlled</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Bundle logic used in this workbook</t>
         </is>
@@ -46334,6 +46742,13 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>14) Use generate_all_possible_bundles.py to produce all bundle combinations up to 3 products.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Select top bundles with no repeated products
Co-authored-by: bassemmamdouh-crypto <bassemmamdouh-crypto@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bundle_planning_template.xlsx
+++ b/bundle_planning_template.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Scoring_Model'!$A$1:$Y$300</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Bundle_Recommendations'!$A$1:$L$300</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'All_Possible_Bundles'!$A$1:$L$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Top_15_Bundles'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Top_15_Bundles'!$A$1:$L$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48188,7 +48188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -48315,488 +48315,8 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>B-000002</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>P-3001</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Aloe Vera Gel 250ml</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>P-2001</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Dry Fruit Mix 200g</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Mixed Category</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>0.7875000000000001</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>0.09000000000000001</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Moves two medium/slow movers with one strong anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>B-000003</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>P-2001</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Dry Fruit Mix 200g</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Same Category</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>0.7375</v>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>0.09000000000000001</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Moves one medium/slow mover using one strong anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>B-000004</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>P-3001</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Aloe Vera Gel 250ml</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>P-1002</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Premium Coffee Beans 1kg</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Mixed Category</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>0.7350000000000001</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Moves two medium/slow movers with one strong anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>B-000005</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>P-2001</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Dry Fruit Mix 200g</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>P-1002</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Premium Coffee Beans 1kg</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Mixed Category</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>0.6675</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>0.09000000000000001</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Moves two medium/slow movers with one strong anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>B-000006</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>3</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>P-3001</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Aloe Vera Gel 250ml</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>P-1001</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Sparkling Water 330ml</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Mixed Category</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>0.651875</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Moves two medium/slow movers with one strong anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>B-000007</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>P-1002</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Premium Coffee Beans 1kg</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Cross Category</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Moves one medium/slow mover using one strong anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>B-000008</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>3</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>P-2001</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Dry Fruit Mix 200g</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>P-1001</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Sparkling Water 330ml</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Mixed Category</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>0.5843750000000001</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Moves two medium/slow movers with one strong anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>B-000009</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>P-1002</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Premium Coffee Beans 1kg</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>P-1001</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Sparkling Water 330ml</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Mixed Category</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="n">
-        <v>0.516875</v>
-      </c>
-      <c r="K10" s="2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Moves two medium/slow movers with one strong anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>B-000010</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>P-2002</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Sea Salt Crackers</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>P-1001</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Sparkling Water 330ml</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Cross Category</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="n">
-        <v>0.446875</v>
-      </c>
-      <c r="K11" s="2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Moves one medium/slow mover using one strong anchor</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>